<commit_message>
refactor: Enhance color handling and camp configuration in gameplay
- Added NewColor32 method to ExternalTypeUtil for converting GameConfig.color32 to Unity's Color32.
- Updated camp configuration to use color32 type instead of string for better color management.
- Modified gameplay camp JSON files to reflect new color structure, improving data consistency.
- Adjusted CampConfig class to deserialize color as Color32, enhancing type safety and clarity.
- Refactored marble initialization to set camp color dynamically based on configuration, improving visual representation in gameplay.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/camp.xlsx
+++ b/Configs/GameConfig/Datas/camp.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
   <si>
     <t>##var</t>
   </si>
@@ -67,6 +67,9 @@
     <t>string</t>
   </si>
   <si>
+    <t>color32</t>
+  </si>
+  <si>
     <t>int</t>
   </si>
   <si>
@@ -79,7 +82,7 @@
     <t>人类</t>
   </si>
   <si>
-    <t>#FFFFFFFF</t>
+    <t>255,255,255,255</t>
   </si>
   <si>
     <t>lancer</t>
@@ -92,6 +95,15 @@
   </si>
   <si>
     <t>archer</t>
+  </si>
+  <si>
+    <t>hollow</t>
+  </si>
+  <si>
+    <t>虚空</t>
+  </si>
+  <si>
+    <t>103,123,255,255</t>
   </si>
 </sst>
 </file>
@@ -748,7 +760,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -764,23 +776,32 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -788,10 +809,16 @@
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -800,7 +827,13 @@
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -809,14 +842,17 @@
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1129,240 +1165,255 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
     <col min="2" max="2" width="25.0909090909091" style="5" customWidth="1"/>
     <col min="3" max="3" width="14.2727272727273" style="5" customWidth="1"/>
     <col min="4" max="4" width="14" style="5" customWidth="1"/>
-    <col min="5" max="5" width="11.5454545454545" style="5" customWidth="1"/>
-    <col min="6" max="6" width="16.4545454545455" style="5" customWidth="1"/>
-    <col min="7" max="7" width="20.1818181818182" style="6" customWidth="1"/>
-    <col min="8" max="8" width="9" style="6"/>
-    <col min="9" max="10" width="17.7272727272727" style="6" customWidth="1"/>
-    <col min="11" max="14" width="9" style="6"/>
+    <col min="5" max="5" width="18.9090909090909" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.4545454545455" style="6" customWidth="1"/>
+    <col min="7" max="7" width="20.1818181818182" style="7" customWidth="1"/>
+    <col min="8" max="8" width="9" style="7"/>
+    <col min="9" max="10" width="17.7272727272727" style="7" customWidth="1"/>
+    <col min="11" max="11" width="9" style="7"/>
+    <col min="12" max="14" width="9" style="8"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:14">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="11" t="s">
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:14">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="11" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:14">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
     </row>
     <row r="4" s="2" customFormat="1" spans="1:14">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="13" t="s">
+      <c r="E4" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="14"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-      <c r="M4" s="15"/>
-      <c r="N4" s="15"/>
+      <c r="F4" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="18"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
     </row>
     <row r="5" s="3" customFormat="1" spans="1:14">
-      <c r="A5" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
+      <c r="A5" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="21"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="25"/>
     </row>
     <row r="6" s="3" customFormat="1" spans="1:14">
-      <c r="A6" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
+      <c r="A6" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="25"/>
+      <c r="N6" s="25"/>
     </row>
     <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:14">
-      <c r="A7" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
+      <c r="A7" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="26"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="29"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
+      <c r="L7" s="30"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="30"/>
     </row>
     <row r="8" spans="1:14">
-      <c r="A8" s="22"/>
-      <c r="B8" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="C8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1000</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="7">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" s="5">
-        <v>1000</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="6">
-        <v>0</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="22" t="s">
-        <v>18</v>
+      <c r="J8" s="6" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="22"/>
-      <c r="B9" s="22"/>
-      <c r="G9" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="6">
+      <c r="G9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" s="7">
         <v>0</v>
       </c>
-      <c r="I9" s="6" t="s">
-        <v>14</v>
+      <c r="I9" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:14">
-      <c r="G10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" s="6">
+      <c r="G10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="7">
         <v>0</v>
       </c>
-      <c r="I10" s="6" t="s">
-        <v>14</v>
+      <c r="I10" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:14">
-      <c r="G11" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" s="6">
+      <c r="G11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="7">
         <v>0</v>
       </c>
-      <c r="I11" s="6" t="s">
-        <v>14</v>
+      <c r="I11" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="B12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="6">
+        <v>1000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>